<commit_message>
docs: add GW-A11Y-43 collapsed menu keyboard focus order defect
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log.xlsx
+++ b/docs/GlobeWest_Remediation_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -796,7 +796,7 @@
         <v>Darken gray labels in the price calculation sidebar.</v>
       </c>
       <c r="G17" t="str">
-        <v>VERIFIED FIXED</v>
+        <v>PENDING REMEDIATION</v>
       </c>
     </row>
     <row r="18">
@@ -888,7 +888,7 @@
         <v>Increase color depth of form validation messages.</v>
       </c>
       <c r="G21" t="str">
-        <v>VERIFIED FIXED</v>
+        <v>PENDING REMEDIATION</v>
       </c>
     </row>
     <row r="22">
@@ -1049,7 +1049,7 @@
         <v>Ensure upload input/button has valid label connection or aria-label.</v>
       </c>
       <c r="G28" t="str">
-        <v>PENDING REMEDIATION</v>
+        <v>VERIFIED FIXED</v>
       </c>
     </row>
     <row r="29">
@@ -1397,9 +1397,32 @@
         <v>PENDING REMEDIATION</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>GW-A11Y-43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>1. Homepage</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2.4.3 Focus Order</v>
+      </c>
+      <c r="D44" t="str">
+        <v>keyboard-navigation</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Collapsed header navigation dropdown sub-links remain focusable in the DOM.</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Apply display: none or visibility: hidden to collapsed submenu containers when closed.</v>
+      </c>
+      <c r="G44" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G44"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: verify 5 PDP and Blog page defects as fixed in remediation log
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log.xlsx
+++ b/docs/GlobeWest_Remediation_Log.xlsx
@@ -796,7 +796,7 @@
         <v>Darken gray labels in the price calculation sidebar.</v>
       </c>
       <c r="G17" t="str">
-        <v>PENDING REMEDIATION</v>
+        <v>VERIFIED FIXED</v>
       </c>
     </row>
     <row r="18">
@@ -888,7 +888,7 @@
         <v>Increase color depth of form validation messages.</v>
       </c>
       <c r="G21" t="str">
-        <v>PENDING REMEDIATION</v>
+        <v>VERIFIED FIXED</v>
       </c>
     </row>
     <row r="22">
@@ -1417,7 +1417,7 @@
         <v>Apply display: none or visibility: hidden to collapsed submenu containers when closed.</v>
       </c>
       <c r="G44" t="str">
-        <v>PENDING REMEDIATION</v>
+        <v>VERIFIED FIXED</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add GW-A11Y-44 invalid ARIA nesting tablist defect
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log.xlsx
+++ b/docs/GlobeWest_Remediation_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -1420,9 +1420,32 @@
         <v>VERIFIED FIXED</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>GW-A11Y-44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>3. PDP (Product Detail)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>1.3.1 Info and Relationships</v>
+      </c>
+      <c r="D45" t="str">
+        <v>aria-allowed-children</v>
+      </c>
+      <c r="E45" t="str">
+        <v>The tablist container nests tabpanel elements directly inside it.</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Move tabpanel elements outside or adjacent to the role=tablist container.</v>
+      </c>
+      <c r="G45" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add GW-A11Y-45 heading-one and GW-A11Y-46 landmark defects on Search Results page
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log.xlsx
+++ b/docs/GlobeWest_Remediation_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:I47"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -1443,9 +1443,61 @@
         <v>PENDING REMEDIATION</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>GW-A11Y-45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>7. Search Results</v>
+      </c>
+      <c r="C46" t="str">
+        <v>1.3.1 Info and Relationships</v>
+      </c>
+      <c r="D46" t="str">
+        <v>page-has-heading-one</v>
+      </c>
+      <c r="E46" t="str">
+        <v>The Search Results page template lacks a semantic level-one heading (h1) tag.</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Add an h1 tag displaying the active search query to identify the page topic.</v>
+      </c>
+      <c r="G46" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>GW-A11Y-46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>7. Search Results</v>
+      </c>
+      <c r="C47" t="str">
+        <v>1.3.1 Info and Relationships</v>
+      </c>
+      <c r="D47" t="str">
+        <v>region</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Some content blocks on the Search Results page are placed outside landmark regions.</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Wrap all page content inside semantic header</v>
+      </c>
+      <c r="G47" t="str">
+        <v xml:space="preserve"> main</v>
+      </c>
+      <c r="H47" t="str">
+        <v xml:space="preserve"> or footer elements.</v>
+      </c>
+      <c r="I47" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update GW-A11Y-45 details targeting div.block-title.title container
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log.xlsx
+++ b/docs/GlobeWest_Remediation_Log.xlsx
@@ -1457,10 +1457,10 @@
         <v>page-has-heading-one</v>
       </c>
       <c r="E46" t="str">
-        <v>The Search Results page template lacks a semantic level-one heading (h1) tag.</v>
+        <v>The Search Results page title is coded inside a non-semantic div.block-title.title container and lacks a level-one heading (h1) tag.</v>
       </c>
       <c r="F46" t="str">
-        <v>Add an h1 tag displaying the active search query to identify the page topic.</v>
+        <v>Convert div.block-title.title to an h1 tag or add a semantic h1 displaying the active search query to identify the page topic.</v>
       </c>
       <c r="G46" t="str">
         <v>PENDING REMEDIATION</v>

</xml_diff>